<commit_message>
Atualização automática - 29/06/2026 11:52
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_saida/digitar.xlsx
+++ b/Aplicativos/GAM/bd_saida/digitar.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
@@ -9,12 +9,15 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$S$34</definedName>
+  </definedNames>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="139">
   <si>
     <t>DEPARTAMENTO</t>
   </si>
@@ -79,49 +82,40 @@
     <t>MERCEARIA</t>
   </si>
   <si>
-    <t>PRODUTOS PET</t>
+    <t>PERECIVEIS</t>
   </si>
   <si>
     <t>PERFUMARIA E LIMPEZA</t>
   </si>
   <si>
-    <t>PERECIVEIS</t>
-  </si>
-  <si>
     <t>NICOLAS AUGUSTO P. BORGES</t>
   </si>
   <si>
+    <t>NIDAL TUBASI</t>
+  </si>
+  <si>
+    <t>SANDRO MARTINS VIANNA</t>
+  </si>
+  <si>
     <t>WETER SONNENFELDET</t>
   </si>
   <si>
-    <t>NIDAL TUBASI</t>
-  </si>
-  <si>
     <t>JOAO BATISTA</t>
   </si>
   <si>
-    <t>SANDRO MARTINS VIANNA</t>
-  </si>
-  <si>
     <t>002</t>
   </si>
   <si>
     <t>003</t>
   </si>
   <si>
-    <t>004</t>
-  </si>
-  <si>
     <t>005</t>
   </si>
   <si>
     <t>006</t>
   </si>
   <si>
-    <t>007</t>
-  </si>
-  <si>
-    <t>011</t>
+    <t>008</t>
   </si>
   <si>
     <t>013</t>
@@ -133,202 +127,187 @@
     <t>017</t>
   </si>
   <si>
-    <t>385</t>
-  </si>
-  <si>
-    <t>389</t>
-  </si>
-  <si>
-    <t>764</t>
-  </si>
-  <si>
-    <t>903</t>
-  </si>
-  <si>
-    <t>1288</t>
-  </si>
-  <si>
-    <t>2814</t>
-  </si>
-  <si>
-    <t>3251</t>
-  </si>
-  <si>
-    <t>4039</t>
-  </si>
-  <si>
-    <t>5172</t>
-  </si>
-  <si>
-    <t>6791</t>
-  </si>
-  <si>
-    <t>17566</t>
-  </si>
-  <si>
-    <t>20611</t>
-  </si>
-  <si>
-    <t>20613</t>
+    <t>018</t>
+  </si>
+  <si>
+    <t>102</t>
+  </si>
+  <si>
+    <t>2100</t>
+  </si>
+  <si>
+    <t>2101</t>
+  </si>
+  <si>
+    <t>2320</t>
+  </si>
+  <si>
+    <t>2519</t>
+  </si>
+  <si>
+    <t>6783</t>
+  </si>
+  <si>
+    <t>1486</t>
+  </si>
+  <si>
+    <t>1606</t>
+  </si>
+  <si>
+    <t>2096</t>
+  </si>
+  <si>
+    <t>2379</t>
+  </si>
+  <si>
+    <t>3153</t>
+  </si>
+  <si>
+    <t>3185</t>
+  </si>
+  <si>
+    <t>3712</t>
+  </si>
+  <si>
+    <t>10148</t>
   </si>
   <si>
     <t>23370</t>
   </si>
   <si>
-    <t>2320</t>
+    <t>36616</t>
+  </si>
+  <si>
+    <t>10144</t>
+  </si>
+  <si>
+    <t>10178</t>
+  </si>
+  <si>
+    <t>1949</t>
+  </si>
+  <si>
+    <t>3911</t>
+  </si>
+  <si>
+    <t>35687</t>
   </si>
   <si>
     <t>2398</t>
   </si>
   <si>
-    <t>3654</t>
-  </si>
-  <si>
-    <t>6783</t>
-  </si>
-  <si>
-    <t>23212</t>
-  </si>
-  <si>
-    <t>33255</t>
-  </si>
-  <si>
-    <t>2140</t>
-  </si>
-  <si>
-    <t>784</t>
-  </si>
-  <si>
-    <t>6782</t>
-  </si>
-  <si>
-    <t>904</t>
-  </si>
-  <si>
-    <t>2150</t>
-  </si>
-  <si>
-    <t>AGUARD 51 VD 965ML</t>
-  </si>
-  <si>
-    <t>ENERG MONSTER LT 473ML GREEN</t>
-  </si>
-  <si>
-    <t>REFRIG COCA COLA PET 200ML ZERO</t>
-  </si>
-  <si>
-    <t>REFRIG PEPSI BLACK LT 350ML</t>
-  </si>
-  <si>
-    <t>CHOC BARRA NESTLE 80G CLASSIC DUO</t>
-  </si>
-  <si>
-    <t>POLENTA PERDIZ 500G INST TEMP</t>
-  </si>
-  <si>
-    <t>SALG KEVYTOS SHOW 38G CEBOLA</t>
-  </si>
-  <si>
-    <t>ALIM GATO BIFFE CAT 1KG ESPECIAL</t>
-  </si>
-  <si>
-    <t>CORANTE TINGECOR 40G GUARANY MARINHO N16</t>
-  </si>
-  <si>
-    <t>LEITE UHT PET ELEGE 1L DESNATADO</t>
-  </si>
-  <si>
-    <t>ENERG RED BULL LT 250ML MELAO MARACUJA</t>
-  </si>
-  <si>
-    <t>MASSA SEMOLA GERMANI 1KG ESPAG</t>
-  </si>
-  <si>
-    <t>MAS ESPAGUETINI ISABELA SEMOLA 500G</t>
+    <t>4202</t>
+  </si>
+  <si>
+    <t>CERV ANTARCTICA SUBZERO GF 1L RETORNAVEL</t>
+  </si>
+  <si>
+    <t>ARROZ BCO SANO OURO TP1 2KG</t>
+  </si>
+  <si>
+    <t>ARROZ BCO REQUINTE TP1 2KG</t>
+  </si>
+  <si>
+    <t>FEIJAO CARIOCA CALDO OURO 1KG</t>
+  </si>
+  <si>
+    <t>KETCHUP HELLMANNS BISN 380G TRAD</t>
+  </si>
+  <si>
+    <t>LEITE UHT TIROL C TAMPA 1L INTEGRAL</t>
+  </si>
+  <si>
+    <t>BISC RECH PASSATEMPO 130G CHOC</t>
+  </si>
+  <si>
+    <t>BISC SALG CLUB SOCIAL 6UN 144G ORIGINAL</t>
+  </si>
+  <si>
+    <t>ARROZ BCO SANO TP1 2KG</t>
+  </si>
+  <si>
+    <t>DUETO OLE LT 170G ERVILHA MILHO</t>
+  </si>
+  <si>
+    <t>SALG KEVYTOS 80G BACONYTOS</t>
+  </si>
+  <si>
+    <t>SALG KEVYTOS BATATA ONDULADA 40G</t>
+  </si>
+  <si>
+    <t>MIST P BOLO APTI 400G QUATRO LEITES</t>
+  </si>
+  <si>
+    <t>SAB FARNESE 180G PITAYA FRAMB</t>
   </si>
   <si>
     <t>SALG KRUKS 35G BACON</t>
   </si>
   <si>
-    <t>FEIJAO CARIOCA CALDO OURO 1KG</t>
+    <t>BOMBOM NESTLE ESPECIALIDADES 220G SORTIDOS</t>
+  </si>
+  <si>
+    <t>SAB FARNESE 180G AVEIA ESFOL</t>
+  </si>
+  <si>
+    <t>SABON PALMOLIVE NATURALS 85G KARITE</t>
+  </si>
+  <si>
+    <t>WAFER MINUETO ROLINHO 40G CHOC</t>
+  </si>
+  <si>
+    <t>ABS C ABAS S LIVRE LV8PG7 AD SUAVE</t>
+  </si>
+  <si>
+    <t>DESOD CREME SECRET CLEAR COTT 45G GEL</t>
   </si>
   <si>
     <t>MILHO VERDE ODERICH LT 200G</t>
   </si>
   <si>
-    <t>LEITE COCO MENINA VD 200ML</t>
-  </si>
-  <si>
-    <t>LEITE UHT TIROL C TAMPA 1L INTEGRAL</t>
-  </si>
-  <si>
-    <t>SAL MOIDO 5 ESTRELAS 1KG</t>
-  </si>
-  <si>
-    <t>REFRIG CHARRUA PET 3L GUARANA</t>
-  </si>
-  <si>
-    <t>ARROZ BCO SANO TP1 5KG</t>
-  </si>
-  <si>
-    <t>REFRIG ANTARCTICA GUARANA PET 2L</t>
-  </si>
-  <si>
-    <t>LEITE UHT TIROL C TAMPA 1L DESN</t>
-  </si>
-  <si>
-    <t>REFRIG PEPSI LT 350ML</t>
-  </si>
-  <si>
-    <t>ARROZ BCO REQUINTE TP1 5KG</t>
-  </si>
-  <si>
-    <t>04/10/2024</t>
-  </si>
-  <si>
-    <t>05/10/2024</t>
-  </si>
-  <si>
-    <t>17/10/2024</t>
-  </si>
-  <si>
-    <t>23/10/2024</t>
-  </si>
-  <si>
-    <t>07/11/2024</t>
-  </si>
-  <si>
-    <t>16/12/2024</t>
-  </si>
-  <si>
-    <t>23/12/2024</t>
+    <t>AMAC GIRANDO SOL 2L AZUL</t>
+  </si>
+  <si>
+    <t>23/09/2024</t>
+  </si>
+  <si>
+    <t>04/12/2024</t>
+  </si>
+  <si>
+    <t>07/12/2024</t>
+  </si>
+  <si>
+    <t>10/12/2024</t>
   </si>
   <si>
     <t>26/04/2025</t>
   </si>
   <si>
+    <t>13/11/2024</t>
+  </si>
+  <si>
+    <t>18/11/2024</t>
+  </si>
+  <si>
+    <t>09/12/2024</t>
+  </si>
+  <si>
+    <t>20/12/2024</t>
+  </si>
+  <si>
+    <t>31/12/2024</t>
+  </si>
+  <si>
     <t>20/06/2025</t>
   </si>
   <si>
-    <t>07/12/2024</t>
-  </si>
-  <si>
-    <t>09/12/2024</t>
-  </si>
-  <si>
-    <t>30/12/2024</t>
-  </si>
-  <si>
-    <t>07/07/2025</t>
-  </si>
-  <si>
-    <t>04/12/2024</t>
-  </si>
-  <si>
-    <t>18/10/2024</t>
-  </si>
-  <si>
-    <t>05/12/2024</t>
+    <t>07/02/2026</t>
+  </si>
+  <si>
+    <t>29/11/2024</t>
+  </si>
+  <si>
+    <t>17/01/2026</t>
   </si>
   <si>
     <t>Ativo</t>
@@ -337,112 +316,124 @@
     <t>12</t>
   </si>
   <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>108</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>6</t>
   </si>
   <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>20</t>
+    <t>211</t>
+  </si>
+  <si>
+    <t>246</t>
+  </si>
+  <si>
+    <t>392</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>23925</t>
+  </si>
+  <si>
+    <t>42666</t>
+  </si>
+  <si>
+    <t>223</t>
+  </si>
+  <si>
+    <t>437</t>
+  </si>
+  <si>
+    <t>454</t>
+  </si>
+  <si>
+    <t>319</t>
+  </si>
+  <si>
+    <t>307</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>189</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>1272</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>29097</t>
+  </si>
+  <si>
+    <t>313</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>249</t>
-  </si>
-  <si>
-    <t>586</t>
-  </si>
-  <si>
-    <t>1116</t>
-  </si>
-  <si>
-    <t>598</t>
-  </si>
-  <si>
-    <t>360</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>235</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>142</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>157</t>
-  </si>
-  <si>
-    <t>136</t>
-  </si>
-  <si>
-    <t>902</t>
-  </si>
-  <si>
-    <t>276</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>13994</t>
-  </si>
-  <si>
-    <t>781</t>
-  </si>
-  <si>
-    <t>1296</t>
-  </si>
-  <si>
-    <t>1392</t>
-  </si>
-  <si>
-    <t>28059</t>
-  </si>
-  <si>
-    <t>419</t>
-  </si>
-  <si>
-    <t>1281</t>
-  </si>
-  <si>
-    <t>576</t>
-  </si>
-  <si>
-    <t>1685</t>
-  </si>
-  <si>
-    <t>306</t>
-  </si>
-  <si>
-    <t>253</t>
-  </si>
-  <si>
-    <t>1735</t>
-  </si>
-  <si>
-    <t>23</t>
+    <t>507</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>92</t>
+  </si>
+  <si>
+    <t>1109</t>
+  </si>
+  <si>
+    <t>275</t>
+  </si>
+  <si>
+    <t>20147</t>
+  </si>
+  <si>
+    <t>52</t>
   </si>
 </sst>
 </file>
@@ -490,9 +481,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Escritório">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -530,7 +521,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Escritório">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -600,7 +591,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Escritório">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -776,6 +767,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S34"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
+    <col min="19" max="19" width="13.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:19">
       <c r="A1" t="s">
@@ -838,34 +835,34 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="F2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I2">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="J2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -877,13 +874,13 @@
         <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="O2">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="P2">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="Q2">
         <v>90</v>
@@ -892,184 +889,184 @@
         <v>2</v>
       </c>
       <c r="S2">
-        <v>40</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="G3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I3">
         <v>6</v>
       </c>
       <c r="J3">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="O3">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="P3">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="Q3">
         <v>90</v>
       </c>
       <c r="R3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S3">
-        <v>381</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H4" t="s">
+        <v>99</v>
+      </c>
+      <c r="I4">
+        <v>15</v>
+      </c>
+      <c r="J4">
+        <v>48</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4" t="s">
+        <v>112</v>
+      </c>
+      <c r="O4">
+        <v>61</v>
+      </c>
+      <c r="P4">
         <v>91</v>
       </c>
-      <c r="G4" t="s">
-        <v>105</v>
-      </c>
-      <c r="H4" t="s">
-        <v>106</v>
-      </c>
-      <c r="I4">
-        <v>12</v>
-      </c>
-      <c r="J4">
-        <v>-1</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4" t="s">
-        <v>116</v>
-      </c>
-      <c r="O4">
-        <v>102</v>
-      </c>
-      <c r="P4">
-        <v>114</v>
-      </c>
       <c r="Q4">
         <v>90</v>
       </c>
       <c r="R4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="S4">
-        <v>61.17</v>
+        <v>67.67</v>
       </c>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="G5" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H5" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="I5">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J5">
-        <v>-6</v>
+        <v>11</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="M5">
         <v>0</v>
       </c>
       <c r="N5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O5">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="P5">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="Q5">
         <v>90</v>
       </c>
       <c r="R5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S5">
-        <v>7</v>
+        <v>67.67</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -1077,31 +1074,31 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="G6" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H6" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="I6">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J6">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -1113,22 +1110,22 @@
         <v>0</v>
       </c>
       <c r="N6" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="O6">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="P6">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="Q6">
         <v>90</v>
       </c>
       <c r="R6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S6">
-        <v>28.06</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -1136,58 +1133,58 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F7" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="G7" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H7" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="I7">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J7">
+        <v>-14</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7" t="s">
+        <v>118</v>
+      </c>
+      <c r="O7">
+        <v>31</v>
+      </c>
+      <c r="P7">
+        <v>46</v>
+      </c>
+      <c r="Q7">
+        <v>90</v>
+      </c>
+      <c r="R7">
         <v>4</v>
       </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7" t="s">
-        <v>119</v>
-      </c>
-      <c r="O7">
-        <v>8</v>
-      </c>
-      <c r="P7">
-        <v>20</v>
-      </c>
-      <c r="Q7">
-        <v>90</v>
-      </c>
-      <c r="R7">
-        <v>2</v>
-      </c>
       <c r="S7">
-        <v>11</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -1195,31 +1192,31 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G8" t="s">
+        <v>97</v>
+      </c>
+      <c r="H8" t="s">
+        <v>102</v>
+      </c>
+      <c r="I8">
         <v>70</v>
       </c>
-      <c r="F8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G8" t="s">
-        <v>105</v>
-      </c>
-      <c r="H8" t="s">
-        <v>109</v>
-      </c>
-      <c r="I8">
-        <v>20</v>
-      </c>
       <c r="J8">
-        <v>-17</v>
+        <v>26</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -1231,54 +1228,54 @@
         <v>0</v>
       </c>
       <c r="N8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="O8">
         <v>48</v>
       </c>
       <c r="P8">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="Q8">
         <v>90</v>
       </c>
       <c r="R8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S8">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:19">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F9" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G9" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H9" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="I9">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="J9">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -1290,13 +1287,13 @@
         <v>0</v>
       </c>
       <c r="N9" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="O9">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="P9">
-        <v>20</v>
+        <v>72</v>
       </c>
       <c r="Q9">
         <v>90</v>
@@ -1305,63 +1302,63 @@
         <v>2</v>
       </c>
       <c r="S9">
-        <v>83.75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:19">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G10" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I10">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="J10">
-        <v>3</v>
+        <v>-133</v>
       </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M10">
         <v>0</v>
       </c>
       <c r="N10" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="O10">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="P10">
-        <v>18</v>
+        <v>126</v>
       </c>
       <c r="Q10">
         <v>90</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S10">
         <v>5</v>
@@ -1369,52 +1366,52 @@
     </row>
     <row r="11" spans="1:19">
       <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
-        <v>29</v>
-      </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="G11" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H11" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="I11">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J11">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M11">
         <v>0</v>
       </c>
       <c r="N11" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="O11">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="P11">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="Q11">
         <v>90</v>
@@ -1423,39 +1420,39 @@
         <v>4</v>
       </c>
       <c r="S11">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:19">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G12" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H12" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -1464,13 +1461,13 @@
         <v>0</v>
       </c>
       <c r="M12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="O12">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P12">
         <v>10</v>
@@ -1479,10 +1476,10 @@
         <v>90</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S12">
-        <v>60.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -1490,31 +1487,31 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="G13" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H13" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="I13">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="J13">
-        <v>25</v>
+        <v>-13</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -1526,13 +1523,13 @@
         <v>0</v>
       </c>
       <c r="N13" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="O13">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="P13">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="Q13">
         <v>90</v>
@@ -1541,7 +1538,7 @@
         <v>3</v>
       </c>
       <c r="S13">
-        <v>5.4</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -1549,31 +1546,31 @@
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="F14" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="G14" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H14" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="I14">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J14">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -1585,22 +1582,22 @@
         <v>0</v>
       </c>
       <c r="N14" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="O14">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="P14">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="Q14">
         <v>90</v>
       </c>
       <c r="R14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14">
-        <v>8</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:19">
@@ -1608,31 +1605,31 @@
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="G15" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H15" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="I15">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J15">
-        <v>-4</v>
+        <v>18</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -1644,22 +1641,22 @@
         <v>0</v>
       </c>
       <c r="N15" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="O15">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="P15">
+        <v>30</v>
+      </c>
+      <c r="Q15">
+        <v>90</v>
+      </c>
+      <c r="R15">
+        <v>12</v>
+      </c>
+      <c r="S15">
         <v>20</v>
-      </c>
-      <c r="Q15">
-        <v>90</v>
-      </c>
-      <c r="R15">
-        <v>2</v>
-      </c>
-      <c r="S15">
-        <v>24.8</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -1667,31 +1664,31 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
         <v>30</v>
       </c>
       <c r="D16" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="G16" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H16" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="I16">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -1703,22 +1700,22 @@
         <v>0</v>
       </c>
       <c r="N16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="O16">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="P16">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="Q16">
         <v>90</v>
       </c>
       <c r="R16">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="S16">
-        <v>42</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:19">
@@ -1726,58 +1723,58 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" t="s">
+        <v>64</v>
+      </c>
+      <c r="F17" t="s">
+        <v>86</v>
+      </c>
+      <c r="G17" t="s">
+        <v>97</v>
+      </c>
+      <c r="H17" t="s">
+        <v>101</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>17</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17" t="s">
+        <v>128</v>
+      </c>
+      <c r="O17">
+        <v>21</v>
+      </c>
+      <c r="P17">
         <v>30</v>
       </c>
-      <c r="D17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" t="s">
-        <v>79</v>
-      </c>
-      <c r="F17" t="s">
-        <v>99</v>
-      </c>
-      <c r="G17" t="s">
-        <v>105</v>
-      </c>
-      <c r="H17" t="s">
-        <v>113</v>
-      </c>
-      <c r="I17">
-        <v>24</v>
-      </c>
-      <c r="J17">
-        <v>182</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17" t="s">
-        <v>127</v>
-      </c>
-      <c r="O17">
-        <v>192</v>
-      </c>
-      <c r="P17">
-        <v>288</v>
-      </c>
       <c r="Q17">
         <v>90</v>
       </c>
       <c r="R17">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="S17">
-        <v>136.88</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -1785,149 +1782,149 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E18" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="F18" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="G18" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H18" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18" t="s">
+        <v>101</v>
+      </c>
+      <c r="O18">
+        <v>13</v>
+      </c>
+      <c r="P18">
+        <v>20</v>
+      </c>
+      <c r="Q18">
+        <v>90</v>
+      </c>
+      <c r="R18">
         <v>24</v>
       </c>
-      <c r="J18">
-        <v>12</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>24</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18" t="s">
-        <v>128</v>
-      </c>
-      <c r="O18">
-        <v>46</v>
-      </c>
-      <c r="P18">
-        <v>70</v>
-      </c>
-      <c r="Q18">
-        <v>90</v>
-      </c>
-      <c r="R18">
-        <v>2</v>
-      </c>
       <c r="S18">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:19">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E19" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F19" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="G19" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H19" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="I19">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J19">
-        <v>-3</v>
+        <v>1341</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="M19">
         <v>0</v>
       </c>
       <c r="N19" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="O19">
-        <v>22</v>
+        <v>2040</v>
       </c>
       <c r="P19">
-        <v>34</v>
+        <v>3060</v>
       </c>
       <c r="Q19">
         <v>90</v>
       </c>
       <c r="R19">
-        <v>3</v>
+        <v>170</v>
       </c>
       <c r="S19">
-        <v>5</v>
+        <v>10749.83</v>
       </c>
     </row>
     <row r="20" spans="1:19">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E20" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="F20" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="G20" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H20" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="I20">
         <v>12</v>
       </c>
       <c r="J20">
-        <v>725</v>
+        <v>4430</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -1939,140 +1936,140 @@
         <v>0</v>
       </c>
       <c r="N20" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="O20">
-        <v>1020</v>
+        <v>5100</v>
       </c>
       <c r="P20">
-        <v>2040</v>
+        <v>6120</v>
       </c>
       <c r="Q20">
         <v>90</v>
       </c>
       <c r="R20">
-        <v>110</v>
+        <v>170</v>
       </c>
       <c r="S20">
-        <v>10945.83</v>
+        <v>10749.83</v>
       </c>
     </row>
     <row r="21" spans="1:19">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s">
         <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D21" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E21" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="F21" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="G21" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H21" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="I21">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J21">
-        <v>63</v>
+        <v>1928</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21">
-        <v>40</v>
+        <v>1032</v>
       </c>
       <c r="M21">
         <v>0</v>
       </c>
       <c r="N21" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="O21">
-        <v>120</v>
+        <v>3060</v>
       </c>
       <c r="P21">
-        <v>180</v>
+        <v>4080</v>
       </c>
       <c r="Q21">
         <v>90</v>
       </c>
       <c r="R21">
-        <v>8</v>
+        <v>85</v>
       </c>
       <c r="S21">
-        <v>1559.4</v>
+        <v>10749.83</v>
       </c>
     </row>
     <row r="22" spans="1:19">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D22" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="E22" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="F22" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="G22" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H22" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="I22">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J22">
-        <v>53</v>
+        <v>3023</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
       <c r="L22">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="M22">
         <v>0</v>
       </c>
       <c r="N22" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="O22">
-        <v>118</v>
+        <v>3060</v>
       </c>
       <c r="P22">
-        <v>154</v>
+        <v>4080</v>
       </c>
       <c r="Q22">
         <v>90</v>
       </c>
       <c r="R22">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="S22">
-        <v>38</v>
+        <v>10749.83</v>
       </c>
     </row>
     <row r="23" spans="1:19">
@@ -2080,31 +2077,31 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E23" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F23" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G23" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H23" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="I23">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="J23">
-        <v>64</v>
+        <v>187</v>
       </c>
       <c r="K23">
         <v>0</v>
@@ -2116,54 +2113,54 @@
         <v>0</v>
       </c>
       <c r="N23" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="O23">
-        <v>88</v>
+        <v>192</v>
       </c>
       <c r="P23">
-        <v>112</v>
+        <v>288</v>
       </c>
       <c r="Q23">
         <v>90</v>
       </c>
       <c r="R23">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="S23">
-        <v>55</v>
+        <v>131.88</v>
       </c>
     </row>
     <row r="24" spans="1:19">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F24" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G24" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H24" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="I24">
         <v>12</v>
       </c>
       <c r="J24">
-        <v>3056</v>
+        <v>2</v>
       </c>
       <c r="K24">
         <v>0</v>
@@ -2175,140 +2172,140 @@
         <v>0</v>
       </c>
       <c r="N24" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="O24">
-        <v>3060</v>
+        <v>10</v>
       </c>
       <c r="P24">
-        <v>4080</v>
+        <v>22</v>
       </c>
       <c r="Q24">
         <v>90</v>
       </c>
       <c r="R24">
-        <v>86</v>
+        <v>2</v>
       </c>
       <c r="S24">
-        <v>10945.83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:19">
       <c r="A25" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" t="s">
+        <v>87</v>
+      </c>
+      <c r="G25" t="s">
+        <v>97</v>
+      </c>
+      <c r="H25" t="s">
+        <v>105</v>
+      </c>
+      <c r="I25">
+        <v>36</v>
+      </c>
+      <c r="J25">
         <v>60</v>
       </c>
-      <c r="E25" t="s">
-        <v>85</v>
-      </c>
-      <c r="F25" t="s">
-        <v>103</v>
-      </c>
-      <c r="G25" t="s">
-        <v>105</v>
-      </c>
-      <c r="H25" t="s">
-        <v>110</v>
-      </c>
-      <c r="I25">
-        <v>8</v>
-      </c>
-      <c r="J25">
-        <v>0</v>
-      </c>
       <c r="K25">
         <v>0</v>
       </c>
       <c r="L25">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="M25">
         <v>0</v>
       </c>
       <c r="N25" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="O25">
-        <v>18</v>
+        <v>198</v>
       </c>
       <c r="P25">
-        <v>30</v>
+        <v>306</v>
       </c>
       <c r="Q25">
         <v>90</v>
       </c>
       <c r="R25">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S25">
-        <v>15.38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:19">
       <c r="A26" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E26" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="F26" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="G26" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" t="s">
         <v>105</v>
       </c>
-      <c r="H26" t="s">
-        <v>107</v>
-      </c>
       <c r="I26">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="J26">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="K26">
         <v>0</v>
       </c>
       <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="N26" t="s">
+        <v>125</v>
+      </c>
+      <c r="O26">
+        <v>132</v>
+      </c>
+      <c r="P26">
+        <v>204</v>
+      </c>
+      <c r="Q26">
+        <v>90</v>
+      </c>
+      <c r="R26">
+        <v>4</v>
+      </c>
+      <c r="S26">
         <v>36</v>
-      </c>
-      <c r="M26">
-        <v>0</v>
-      </c>
-      <c r="N26" t="s">
-        <v>136</v>
-      </c>
-      <c r="O26">
-        <v>118</v>
-      </c>
-      <c r="P26">
-        <v>154</v>
-      </c>
-      <c r="Q26">
-        <v>90</v>
-      </c>
-      <c r="R26">
-        <v>9</v>
-      </c>
-      <c r="S26">
-        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:19">
@@ -2319,34 +2316,34 @@
         <v>27</v>
       </c>
       <c r="C27" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D27" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E27" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F27" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="G27" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H27" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I27">
-        <v>6</v>
+        <v>108</v>
       </c>
       <c r="J27">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="K27">
         <v>0</v>
       </c>
       <c r="L27">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="M27">
         <v>0</v>
@@ -2355,110 +2352,110 @@
         <v>106</v>
       </c>
       <c r="O27">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="P27">
-        <v>34</v>
+        <v>174</v>
       </c>
       <c r="Q27">
         <v>90</v>
       </c>
       <c r="R27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S27">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:19">
       <c r="A28" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B28" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" t="s">
+        <v>47</v>
+      </c>
+      <c r="E28" t="s">
+        <v>70</v>
+      </c>
+      <c r="F28" t="s">
+        <v>91</v>
+      </c>
+      <c r="G28" t="s">
+        <v>97</v>
+      </c>
+      <c r="H28" t="s">
+        <v>100</v>
+      </c>
+      <c r="I28">
+        <v>10</v>
+      </c>
+      <c r="J28">
+        <v>10</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>10</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28" t="s">
+        <v>122</v>
+      </c>
+      <c r="O28">
         <v>24</v>
       </c>
-      <c r="C28" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28" t="s">
-        <v>60</v>
-      </c>
-      <c r="E28" t="s">
-        <v>85</v>
-      </c>
-      <c r="F28" t="s">
-        <v>103</v>
-      </c>
-      <c r="G28" t="s">
-        <v>105</v>
-      </c>
-      <c r="H28" t="s">
-        <v>110</v>
-      </c>
-      <c r="I28">
-        <v>8</v>
-      </c>
-      <c r="J28">
-        <v>-4</v>
-      </c>
-      <c r="K28">
-        <v>0</v>
-      </c>
-      <c r="L28">
-        <v>16</v>
-      </c>
-      <c r="M28">
-        <v>0</v>
-      </c>
-      <c r="N28" t="s">
-        <v>137</v>
-      </c>
-      <c r="O28">
-        <v>72</v>
-      </c>
       <c r="P28">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="Q28">
         <v>90</v>
       </c>
       <c r="R28">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="S28">
-        <v>15.38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:19">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D29" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E29" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="F29" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="G29" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H29" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I29">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="J29">
-        <v>116</v>
+        <v>1</v>
       </c>
       <c r="K29">
         <v>0</v>
@@ -2470,72 +2467,72 @@
         <v>0</v>
       </c>
       <c r="N29" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="O29">
-        <v>120</v>
+        <v>22</v>
       </c>
       <c r="P29">
-        <v>168</v>
+        <v>52</v>
       </c>
       <c r="Q29">
         <v>90</v>
       </c>
       <c r="R29">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S29">
-        <v>355</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:19">
       <c r="A30" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" t="s">
+        <v>51</v>
+      </c>
+      <c r="E30" t="s">
+        <v>74</v>
+      </c>
+      <c r="F30" t="s">
+        <v>93</v>
+      </c>
+      <c r="G30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H30" t="s">
+        <v>100</v>
+      </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
+      <c r="J30">
+        <v>-1</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30" t="s">
+        <v>126</v>
+      </c>
+      <c r="O30">
         <v>24</v>
       </c>
-      <c r="C30" t="s">
-        <v>37</v>
-      </c>
-      <c r="D30" t="s">
-        <v>62</v>
-      </c>
-      <c r="E30" t="s">
-        <v>87</v>
-      </c>
-      <c r="F30" t="s">
-        <v>92</v>
-      </c>
-      <c r="G30" t="s">
-        <v>105</v>
-      </c>
-      <c r="H30" t="s">
-        <v>106</v>
-      </c>
-      <c r="I30">
-        <v>12</v>
-      </c>
-      <c r="J30">
-        <v>17</v>
-      </c>
-      <c r="K30">
-        <v>0</v>
-      </c>
-      <c r="L30">
-        <v>0</v>
-      </c>
-      <c r="M30">
-        <v>0</v>
-      </c>
-      <c r="N30" t="s">
-        <v>139</v>
-      </c>
-      <c r="O30">
-        <v>32</v>
-      </c>
       <c r="P30">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="Q30">
         <v>90</v>
@@ -2544,57 +2541,57 @@
         <v>4</v>
       </c>
       <c r="S30">
-        <v>7</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="31" spans="1:19">
       <c r="A31" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s">
+        <v>33</v>
+      </c>
+      <c r="D31" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" t="s">
+        <v>78</v>
+      </c>
+      <c r="F31" t="s">
+        <v>95</v>
+      </c>
+      <c r="G31" t="s">
+        <v>97</v>
+      </c>
+      <c r="H31" t="s">
+        <v>101</v>
+      </c>
+      <c r="I31">
         <v>24</v>
       </c>
-      <c r="C31" t="s">
-        <v>38</v>
-      </c>
-      <c r="D31" t="s">
-        <v>62</v>
-      </c>
-      <c r="E31" t="s">
-        <v>87</v>
-      </c>
-      <c r="F31" t="s">
-        <v>92</v>
-      </c>
-      <c r="G31" t="s">
-        <v>105</v>
-      </c>
-      <c r="H31" t="s">
-        <v>106</v>
-      </c>
-      <c r="I31">
-        <v>12</v>
-      </c>
       <c r="J31">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="K31">
         <v>0</v>
       </c>
       <c r="L31">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M31">
         <v>0</v>
       </c>
       <c r="N31" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="O31">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="P31">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="Q31">
         <v>90</v>
@@ -2603,7 +2600,7 @@
         <v>3</v>
       </c>
       <c r="S31">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:19">
@@ -2614,28 +2611,28 @@
         <v>26</v>
       </c>
       <c r="C32" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D32" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E32" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F32" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="G32" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H32" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="I32">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="J32">
-        <v>131</v>
+        <v>19</v>
       </c>
       <c r="K32">
         <v>0</v>
@@ -2644,25 +2641,25 @@
         <v>0</v>
       </c>
       <c r="M32">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="N32" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="O32">
-        <v>184</v>
+        <v>26</v>
       </c>
       <c r="P32">
-        <v>280</v>
+        <v>50</v>
       </c>
       <c r="Q32">
         <v>90</v>
       </c>
       <c r="R32">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="S32">
-        <v>53</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:19">
@@ -2670,120 +2667,125 @@
         <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C33" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D33" t="s">
         <v>55</v>
       </c>
       <c r="E33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F33" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G33" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H33" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="I33">
         <v>24</v>
       </c>
       <c r="J33">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="K33">
         <v>0</v>
       </c>
       <c r="L33">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="M33">
         <v>0</v>
       </c>
       <c r="N33" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="O33">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="P33">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="Q33">
         <v>90</v>
       </c>
       <c r="R33">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S33">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:19">
       <c r="A34" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C34" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D34" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="E34" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G34" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H34" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="I34">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="J34">
+        <v>-1</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34" t="s">
+        <v>138</v>
+      </c>
+      <c r="O34">
+        <v>52</v>
+      </c>
+      <c r="P34">
+        <v>76</v>
+      </c>
+      <c r="Q34">
+        <v>90</v>
+      </c>
+      <c r="R34">
         <v>5</v>
-      </c>
-      <c r="K34">
-        <v>0</v>
-      </c>
-      <c r="L34">
-        <v>6</v>
-      </c>
-      <c r="M34">
-        <v>0</v>
-      </c>
-      <c r="N34" t="s">
-        <v>142</v>
-      </c>
-      <c r="O34">
-        <v>14</v>
-      </c>
-      <c r="P34">
-        <v>26</v>
-      </c>
-      <c r="Q34">
-        <v>90</v>
-      </c>
-      <c r="R34">
-        <v>3</v>
       </c>
       <c r="S34">
         <v>5</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:S34">
+    <sortState ref="A2:S34">
+      <sortCondition ref="E1:E34"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualização automática - 18/09/2026 14:07
</commit_message>
<xml_diff>
--- a/Aplicativos/GAM/bd_saida/digitar.xlsx
+++ b/Aplicativos/GAM/bd_saida/digitar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usr\Downloads\Equipes_Agentes\Aplicativos\GAM\bd_saida\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEDDC212-01B5-477E-BB3A-ECC0B168C605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749973BA-586E-4370-8302-916B19F1F07E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$46</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="234">
   <si>
     <t>DEPARTAMENTO</t>
   </si>
@@ -102,33 +102,30 @@
     <t>Estq_CD_cx</t>
   </si>
   <si>
+    <t>PERECIVEIS</t>
+  </si>
+  <si>
+    <t>MERCEARIA</t>
+  </si>
+  <si>
     <t>BEBIDAS</t>
   </si>
   <si>
-    <t>MERCEARIA</t>
-  </si>
-  <si>
-    <t>PRODUTOS PET</t>
-  </si>
-  <si>
     <t>PERFUMARIA E LIMPEZA</t>
   </si>
   <si>
-    <t>PERECIVEIS</t>
+    <t>SANDRO MARTINS VIANNA</t>
+  </si>
+  <si>
+    <t>NIDAL TUBASI</t>
   </si>
   <si>
     <t>NICOLAS AUGUSTO P. BORGES</t>
   </si>
   <si>
-    <t>NIDAL TUBASI</t>
-  </si>
-  <si>
     <t>JOAO BATISTA</t>
   </si>
   <si>
-    <t>SANDRO MARTINS VIANNA</t>
-  </si>
-  <si>
     <t>WETER SONNENFELDET</t>
   </si>
   <si>
@@ -144,7 +141,13 @@
     <t>004</t>
   </si>
   <si>
-    <t>006</t>
+    <t>005</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t>008</t>
   </si>
   <si>
     <t>011</t>
@@ -153,452 +156,588 @@
     <t>012</t>
   </si>
   <si>
+    <t>013</t>
+  </si>
+  <si>
     <t>014</t>
   </si>
   <si>
     <t>017</t>
   </si>
   <si>
-    <t>018</t>
+    <t>6783</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>6781</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>838</t>
+  </si>
+  <si>
+    <t>5431</t>
+  </si>
+  <si>
+    <t>49</t>
   </si>
   <si>
     <t>795</t>
   </si>
   <si>
+    <t>389</t>
+  </si>
+  <si>
+    <t>10856</t>
+  </si>
+  <si>
+    <t>806</t>
+  </si>
+  <si>
+    <t>1297</t>
+  </si>
+  <si>
+    <t>835</t>
+  </si>
+  <si>
+    <t>910</t>
+  </si>
+  <si>
+    <t>2396</t>
+  </si>
+  <si>
+    <t>5673</t>
+  </si>
+  <si>
+    <t>5678</t>
+  </si>
+  <si>
+    <t>7878</t>
+  </si>
+  <si>
+    <t>10147</t>
+  </si>
+  <si>
+    <t>10148</t>
+  </si>
+  <si>
+    <t>17341</t>
+  </si>
+  <si>
+    <t>17349</t>
+  </si>
+  <si>
+    <t>22999</t>
+  </si>
+  <si>
+    <t>23111</t>
+  </si>
+  <si>
+    <t>33265</t>
+  </si>
+  <si>
+    <t>34977</t>
+  </si>
+  <si>
+    <t>1657</t>
+  </si>
+  <si>
+    <t>1713</t>
+  </si>
+  <si>
+    <t>2499</t>
+  </si>
+  <si>
+    <t>2831</t>
+  </si>
+  <si>
+    <t>2924</t>
+  </si>
+  <si>
+    <t>3475</t>
+  </si>
+  <si>
+    <t>3531</t>
+  </si>
+  <si>
+    <t>13277</t>
+  </si>
+  <si>
+    <t>39236</t>
+  </si>
+  <si>
+    <t>2179</t>
+  </si>
+  <si>
+    <t>2232</t>
+  </si>
+  <si>
+    <t>1575</t>
+  </si>
+  <si>
+    <t>39265</t>
+  </si>
+  <si>
+    <t>LEITE UHT TIROL C TAMP INT 1L</t>
+  </si>
+  <si>
+    <t>AGUA MIN CRYSTAL PET 500ML S GAS</t>
+  </si>
+  <si>
+    <t>LEITE UHT ELEGE INT 1L</t>
+  </si>
+  <si>
+    <t>AGUA MIN CRYSTAL PET 500ML C GAS</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI PET 3L GUARANA</t>
+  </si>
+  <si>
+    <t>DESINF AQUAFAST HARMONIA 5L LAVANDA</t>
+  </si>
+  <si>
+    <t>AGUA MIN FLORESTA PET 500ML S GAS</t>
+  </si>
+  <si>
+    <t>REFRIG COCA COLA PET 2L ZERO</t>
+  </si>
+  <si>
+    <t>ENERG MONSTER LT 473ML GREEN</t>
+  </si>
+  <si>
+    <t>CASTANHA PARA UNIAGRO S CASCA</t>
+  </si>
+  <si>
+    <t>REFRIG FANTA LARANJA PET 2L</t>
+  </si>
+  <si>
+    <t>CHOC BARRA NESTLE 80G CRUNCH</t>
+  </si>
+  <si>
+    <t>REFRIG PET COCA COLA 3L</t>
+  </si>
+  <si>
+    <t>REFRIG SUKITA LT 350 ML</t>
+  </si>
+  <si>
+    <t>MILHO VERDE OLE LT 170G</t>
+  </si>
+  <si>
+    <t>DET LIQ GIRANDO SOL 500ML LIMAO</t>
+  </si>
+  <si>
+    <t>DET LIQ GOTA LIMPA 500ML CRISTAL</t>
+  </si>
+  <si>
+    <t>SABONETE DOVE 90G KARITE BAUNILHA</t>
+  </si>
+  <si>
+    <t>SAB FARNESE 180G LAVANDA MENTA</t>
+  </si>
+  <si>
+    <t>SAB FARNESE 180G PITAYA FRAMB</t>
+  </si>
+  <si>
+    <t>DET LIQ BIO KRISS 500ML NEUTRO</t>
+  </si>
+  <si>
+    <t>DET LIQ GOTA LIMPA 1L NATURAL</t>
+  </si>
+  <si>
+    <t>SAB FONTANA SENSUS 150G AMANHECER PERS</t>
+  </si>
+  <si>
+    <t>SAB PALMOLIVE 85G ARGILA EUCALIP</t>
+  </si>
+  <si>
+    <t>REFRIG FRUKI GUAR ZR PET 3L GUARANA ZERO</t>
+  </si>
+  <si>
+    <t>SAB MARAN SUAVE 80G PESSEGO</t>
+  </si>
+  <si>
+    <t>WAFFER ISABELA 100G DOCE DE LEITE</t>
+  </si>
+  <si>
+    <t>PIPOCA DOCE KEVYTOS 50G</t>
+  </si>
+  <si>
+    <t>KETCHUP ODERICH BISN 400G PICANTE</t>
+  </si>
+  <si>
+    <t>MASSA C OVOS GERMANI 500G ESPAGUETE</t>
+  </si>
+  <si>
+    <t>MASSA C OVOS PARATI 500G RIGATONI</t>
+  </si>
+  <si>
+    <t>TEMP COLORIFICO APTI 100G</t>
+  </si>
+  <si>
+    <t>FERM QUIMICO PO ROYAL PT 100G</t>
+  </si>
+  <si>
+    <t>BISC AGUA SAL ORQUIDEA 665GR</t>
+  </si>
+  <si>
+    <t>CERV AMSTEL ULTRA LN 330ML</t>
+  </si>
+  <si>
+    <t>CHA PRENDA GOLD 15G CIDREIRA</t>
+  </si>
+  <si>
+    <t>CAPSULA DOLCE GUSTO 117G C 10 CAPPUCCINO</t>
+  </si>
+  <si>
+    <t>BISC SALG GERMANI GRISSINI 175G</t>
+  </si>
+  <si>
+    <t>REFRE FRUKITO PET 5L FRUTAS CITRICAS</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>26/04/2025</t>
+  </si>
+  <si>
+    <t>20/06/2025</t>
+  </si>
+  <si>
+    <t>18/09/2024</t>
+  </si>
+  <si>
+    <t>21/10/2024</t>
+  </si>
+  <si>
+    <t>19/09/2024</t>
+  </si>
+  <si>
+    <t>18/10/2024</t>
+  </si>
+  <si>
+    <t>05/10/2024</t>
+  </si>
+  <si>
+    <t>11/06/2025</t>
+  </si>
+  <si>
+    <t>19/10/2024</t>
+  </si>
+  <si>
+    <t>07/11/2024</t>
+  </si>
+  <si>
+    <t>23/10/2024</t>
+  </si>
+  <si>
+    <t>09/12/2024</t>
+  </si>
+  <si>
+    <t>08/07/2025</t>
+  </si>
+  <si>
+    <t>08/12/2025</t>
+  </si>
+  <si>
+    <t>19/11/2024</t>
+  </si>
+  <si>
+    <t>22/11/2024</t>
+  </si>
+  <si>
+    <t>10/12/2024</t>
+  </si>
+  <si>
+    <t>16/12/2024</t>
+  </si>
+  <si>
+    <t>17/12/2024</t>
+  </si>
+  <si>
+    <t>27/12/2024</t>
+  </si>
+  <si>
+    <t>28/12/2024</t>
+  </si>
+  <si>
+    <t>24/08/2026</t>
+  </si>
+  <si>
+    <t>05/12/2024</t>
+  </si>
+  <si>
+    <t>14/11/2024</t>
+  </si>
+  <si>
+    <t>26/08/2026</t>
+  </si>
+  <si>
+    <t>Ativo</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>108</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
     <t>50</t>
   </si>
   <si>
-    <t>835</t>
-  </si>
-  <si>
-    <t>840</t>
-  </si>
-  <si>
-    <t>293</t>
-  </si>
-  <si>
-    <t>3991</t>
-  </si>
-  <si>
-    <t>8840</t>
-  </si>
-  <si>
-    <t>12393</t>
-  </si>
-  <si>
-    <t>17160</t>
-  </si>
-  <si>
-    <t>37423</t>
-  </si>
-  <si>
-    <t>747</t>
-  </si>
-  <si>
-    <t>8288</t>
-  </si>
-  <si>
-    <t>4048</t>
-  </si>
-  <si>
-    <t>10173</t>
-  </si>
-  <si>
-    <t>4000</t>
-  </si>
-  <si>
-    <t>5857</t>
-  </si>
-  <si>
-    <t>6781</t>
-  </si>
-  <si>
-    <t>8702</t>
-  </si>
-  <si>
-    <t>36996</t>
-  </si>
-  <si>
-    <t>20621</t>
-  </si>
-  <si>
-    <t>4052</t>
-  </si>
-  <si>
-    <t>33255</t>
-  </si>
-  <si>
-    <t>39321</t>
-  </si>
-  <si>
-    <t>749</t>
-  </si>
-  <si>
-    <t>3042</t>
-  </si>
-  <si>
-    <t>3617</t>
-  </si>
-  <si>
-    <t>19844</t>
-  </si>
-  <si>
-    <t>22794</t>
-  </si>
-  <si>
-    <t>37047</t>
-  </si>
-  <si>
-    <t>39075</t>
-  </si>
-  <si>
-    <t>39234</t>
-  </si>
-  <si>
-    <t>REFRIG COCA COLA PET 2L ZERO</t>
-  </si>
-  <si>
-    <t>AGUA MIN DA PEDRA PET 5L S GAS</t>
-  </si>
-  <si>
-    <t>REFRIG PET COCA COLA 3L</t>
-  </si>
-  <si>
-    <t>REFRIG PEPSI PET 3L</t>
-  </si>
-  <si>
-    <t>CERV STELLA ARTOIS LN 330ML</t>
-  </si>
-  <si>
-    <t>RACAO DOG CHOW SH 85G MULTI PROTEINAS</t>
-  </si>
-  <si>
-    <t>AMAC AQUAFAST EMB ECON 5L VERM SEDUCAO</t>
-  </si>
-  <si>
-    <t>AMACIANTE AQUAFAST 2L MANHA AZ</t>
-  </si>
-  <si>
-    <t>DESINF AQUAFAST 2L CHA BRANCO</t>
-  </si>
-  <si>
-    <t>DESINF AQUAFAST 2L HARMONIA NAT</t>
-  </si>
-  <si>
-    <t>ACUCAR CRISTAL GASPARIN 2KG</t>
-  </si>
-  <si>
-    <t>SH PANTENE 175ML EQUIL ALGA MAR</t>
-  </si>
-  <si>
-    <t>RACAO FRISKIES SH 85G FGO MOLHO</t>
-  </si>
-  <si>
-    <t>SABON PALMOLIVE NATURALS 85G CAMELIA AMEND</t>
-  </si>
-  <si>
-    <t>RACAO DOG CHOW SH 85G AD CAR FGO SALM</t>
-  </si>
-  <si>
-    <t>ESC DENTAL SORRISO MACIA</t>
-  </si>
-  <si>
-    <t>LEITE UHT ELEGE INT 1L</t>
-  </si>
-  <si>
-    <t>VASSOURA BETTANIN NOVICA RF167</t>
-  </si>
-  <si>
-    <t>FARINHA TAPIOCA ROCHA 500G TRAD</t>
-  </si>
-  <si>
-    <t>MAS FURADINHO ISABELA SEMOLA 400G</t>
-  </si>
-  <si>
-    <t>RACAO FRISKIES SH 85G PERU MOLHO</t>
-  </si>
-  <si>
-    <t>REFRIG CHARRUA PET 3L GUARANA</t>
-  </si>
-  <si>
-    <t>RACAO DOG CHOW SH 85G ALTA PROTEINA</t>
-  </si>
-  <si>
-    <t>REFRIG SARANDI PET 1 5L GUARANA ZERO</t>
-  </si>
-  <si>
-    <t>CEREAL MAT NESTLE CX210G NESCAU DUO</t>
-  </si>
-  <si>
-    <t>GELATINA NEILAR 20G AMORA</t>
-  </si>
-  <si>
-    <t>L MOVEIS POLWAX 200ML JASMIN</t>
-  </si>
-  <si>
-    <t>RATICIDA RATICID GRANULADO 25G</t>
-  </si>
-  <si>
-    <t>FAROFA ROCHA CASEIRA 300GBACON</t>
-  </si>
-  <si>
-    <t>MOLHO TOM SACCIALI 520G PASSATA</t>
-  </si>
-  <si>
-    <t>PALMITO PETRY PUPUNHA PICADO 300G</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>18/10/2024</t>
-  </si>
-  <si>
-    <t>20/06/2025</t>
-  </si>
-  <si>
-    <t>19/09/2024</t>
-  </si>
-  <si>
-    <t>21/10/2024</t>
-  </si>
-  <si>
-    <t>01/10/2024</t>
-  </si>
-  <si>
-    <t>26/04/2025</t>
-  </si>
-  <si>
-    <t>09/03/2026</t>
-  </si>
-  <si>
-    <t>17/10/2024</t>
-  </si>
-  <si>
-    <t>20/02/2026</t>
-  </si>
-  <si>
-    <t>07/07/2025</t>
-  </si>
-  <si>
-    <t>27/08/2026</t>
-  </si>
-  <si>
-    <t>19/12/2024</t>
-  </si>
-  <si>
-    <t>30/12/2024</t>
-  </si>
-  <si>
-    <t>23/02/2026</t>
-  </si>
-  <si>
-    <t>31/07/2026</t>
-  </si>
-  <si>
-    <t>24/08/2026</t>
-  </si>
-  <si>
-    <t>Ativo</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>108</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>480</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>292</t>
+    <t>4038</t>
   </si>
   <si>
     <t>0</t>
   </si>
   <si>
-    <t>250</t>
+    <t>1511</t>
+  </si>
+  <si>
+    <t>1845</t>
+  </si>
+  <si>
+    <t>5962</t>
+  </si>
+  <si>
+    <t>1629</t>
+  </si>
+  <si>
+    <t>73</t>
+  </si>
+  <si>
+    <t>13983</t>
+  </si>
+  <si>
+    <t>1391</t>
+  </si>
+  <si>
+    <t>588</t>
+  </si>
+  <si>
+    <t>,58</t>
+  </si>
+  <si>
+    <t>1081</t>
   </si>
   <si>
     <t>1413</t>
   </si>
   <si>
-    <t>1358</t>
-  </si>
-  <si>
-    <t>562</t>
-  </si>
-  <si>
-    <t>2221</t>
-  </si>
-  <si>
-    <t>63</t>
+    <t>170</t>
+  </si>
+  <si>
+    <t>654</t>
+  </si>
+  <si>
+    <t>1,57</t>
+  </si>
+  <si>
+    <t>315</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>1739</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>418</t>
+  </si>
+  <si>
+    <t>187</t>
+  </si>
+  <si>
+    <t>172</t>
+  </si>
+  <si>
+    <t>158</t>
+  </si>
+  <si>
+    <t>286</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
+    <t>1016</t>
+  </si>
+  <si>
+    <t>35487</t>
+  </si>
+  <si>
+    <t>3068</t>
+  </si>
+  <si>
+    <t>628</t>
+  </si>
+  <si>
+    <t>579</t>
+  </si>
+  <si>
+    <t>210</t>
+  </si>
+  <si>
+    <t>827</t>
+  </si>
+  <si>
+    <t>194</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>1150</t>
+  </si>
+  <si>
+    <t>208</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>139</t>
+  </si>
+  <si>
+    <t>218</t>
   </si>
   <si>
     <t>37</t>
   </si>
   <si>
-    <t>79</t>
-  </si>
-  <si>
-    <t>69</t>
-  </si>
-  <si>
-    <t>54</t>
-  </si>
-  <si>
-    <t>1844</t>
-  </si>
-  <si>
-    <t>1569</t>
-  </si>
-  <si>
-    <t>263</t>
-  </si>
-  <si>
-    <t>123</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>61</t>
-  </si>
-  <si>
-    <t>2899</t>
-  </si>
-  <si>
-    <t>207</t>
-  </si>
-  <si>
-    <t>184</t>
-  </si>
-  <si>
-    <t>299</t>
-  </si>
-  <si>
-    <t>82</t>
-  </si>
-  <si>
-    <t>1502</t>
-  </si>
-  <si>
-    <t>53</t>
-  </si>
-  <si>
-    <t>73</t>
-  </si>
-  <si>
-    <t>114</t>
-  </si>
-  <si>
-    <t>78</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>289</t>
-  </si>
-  <si>
-    <t>52</t>
+    <t>LATICINIOS TIROL LTDA.</t>
   </si>
   <si>
     <t>SPAL IND BRAS BEBIDAS AS</t>
   </si>
   <si>
+    <t>LACTALIS BRASIL COM IMP EXP LTDA</t>
+  </si>
+  <si>
     <t>BEBIDAS FRUKI LTDA</t>
   </si>
   <si>
+    <t>AQUAFAST PROD LIMPEZA/HIGIENE LTDA</t>
+  </si>
+  <si>
+    <t>AGUAS MINERAIS SARANDI LTDA</t>
+  </si>
+  <si>
+    <t>UNIAGRO -IND.E COM.DE PROD.ALIM.LTDA</t>
+  </si>
+  <si>
+    <t>NESTLE BRASIL LTDA</t>
+  </si>
+  <si>
     <t>CRBS AS CDD PELOTAS</t>
   </si>
   <si>
-    <t>NESTLE BRASIL LTDA</t>
-  </si>
-  <si>
-    <t>AQUAFAST PROD LIMPEZA/HIGIENE LTDA</t>
-  </si>
-  <si>
-    <t>GASPARIN CEREAIS LTDA ME</t>
+    <t>ANGELO AURICCHIO &amp; CIA LTDA</t>
+  </si>
+  <si>
+    <t>IND COM PROD LIMP GIRANDO SOL LTDA</t>
+  </si>
+  <si>
+    <t>BERTOLINI INDUSTRIA QUIMICA LTDA</t>
+  </si>
+  <si>
+    <t>ZAFFALON E CIA LTDA</t>
   </si>
   <si>
     <t>ONIZ DISTRIBUID LTDA SCJ</t>
   </si>
   <si>
+    <t>SENIR EMBALAGENS LTDA</t>
+  </si>
+  <si>
+    <t>FONTANA S.A</t>
+  </si>
+  <si>
     <t>UNIDASUL DISTRIBUIDORA ALIMENTICIA S/A</t>
   </si>
   <si>
-    <t>PODAL IND E COM DE ALIMENTOS LTDA</t>
-  </si>
-  <si>
-    <t>LACTALIS BRASIL COM IMP EXP LTDA</t>
-  </si>
-  <si>
-    <t>ROCHA E FILHOS LTDA</t>
+    <t>ATACADAO S.A.</t>
   </si>
   <si>
     <t>M DIAS BRANCO S.A IND E COM DE ALIMENTOS</t>
   </si>
   <si>
-    <t>AGUAS MINERAIS SARANDI LTDA</t>
-  </si>
-  <si>
-    <t>NEILAR IND COM DE ALIMENTOS LTDA</t>
-  </si>
-  <si>
-    <t>POLWAX INDUSTRIA QUIMICA LTDA</t>
-  </si>
-  <si>
-    <t>AGROCOMERCIAL SANDRI LTDA</t>
-  </si>
-  <si>
-    <t>STELLA DORO ALIMENTOS LTDA</t>
-  </si>
-  <si>
-    <t>INDUSTRIA DE ALIMENTOS PETRY LTDA</t>
+    <t>DELAVY ALIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>CONSERVAS ODERICH SA</t>
+  </si>
+  <si>
+    <t>GERMANI ALIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>PARATI IND.COM.DE ALIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>APTI ALIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>TOPFLEX DISTRIBUIDOR DE ALIMENTOS</t>
+  </si>
+  <si>
+    <t>TONDO S/A</t>
+  </si>
+  <si>
+    <t>CARLOS CANCIAN E CIA LTDA</t>
+  </si>
+  <si>
+    <t>CHA PRENDA DO BRASIL IND E COM EIRELI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -626,9 +765,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,83 +1071,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X35"/>
+  <dimension ref="A1:X46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="48" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1018,34 +1156,34 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="F2" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="G2" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="H2" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I2" t="s">
-        <v>125</v>
+        <v>151</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K2">
-        <v>13</v>
+        <v>422</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1057,13 +1195,13 @@
         <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="P2">
-        <v>28</v>
+        <v>480</v>
       </c>
       <c r="Q2">
-        <v>44</v>
+        <v>600</v>
       </c>
       <c r="R2">
         <v>0</v>
@@ -1075,51 +1213,51 @@
         <v>90</v>
       </c>
       <c r="U2">
-        <v>15441</v>
+        <v>15208</v>
       </c>
       <c r="V2" t="s">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="W2">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="X2">
-        <v>157</v>
+        <v>5958</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G3" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="H3" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I3" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="J3">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>40</v>
+        <v>130</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -1131,13 +1269,13 @@
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>138</v>
+        <v>167</v>
       </c>
       <c r="P3">
-        <v>48</v>
+        <v>162</v>
       </c>
       <c r="Q3">
-        <v>72</v>
+        <v>258</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -1149,16 +1287,16 @@
         <v>90</v>
       </c>
       <c r="U3">
-        <v>6424</v>
+        <v>15441</v>
       </c>
       <c r="V3" t="s">
-        <v>168</v>
+        <v>207</v>
       </c>
       <c r="W3">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="X3">
-        <v>535</v>
+        <v>23.08</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
@@ -1166,34 +1304,34 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G4" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="H4" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I4" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="J4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K4">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -1205,13 +1343,13 @@
         <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>139</v>
+        <v>168</v>
       </c>
       <c r="P4">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="Q4">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -1223,51 +1361,51 @@
         <v>90</v>
       </c>
       <c r="U4">
-        <v>15441</v>
+        <v>9379</v>
       </c>
       <c r="V4" t="s">
-        <v>167</v>
+        <v>208</v>
       </c>
       <c r="W4">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="X4">
-        <v>387</v>
+        <v>776</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="F5" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G5" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="H5" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I5" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="K5">
-        <v>153</v>
+        <v>23</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -1279,69 +1417,69 @@
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="P5">
-        <v>156</v>
+        <v>76</v>
       </c>
       <c r="Q5">
-        <v>240</v>
+        <v>112</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>1008</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>1308</v>
       </c>
       <c r="T5">
         <v>90</v>
       </c>
       <c r="U5">
-        <v>9638</v>
+        <v>15441</v>
       </c>
       <c r="V5" t="s">
-        <v>169</v>
+        <v>207</v>
       </c>
       <c r="W5">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="X5">
-        <v>44</v>
+        <v>218.58</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F6" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G6" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="H6" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I6" t="s">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="J6">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>72</v>
+        <v>148</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -1353,13 +1491,13 @@
         <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>141</v>
+        <v>170</v>
       </c>
       <c r="P6">
-        <v>76</v>
+        <v>180</v>
       </c>
       <c r="Q6">
-        <v>124</v>
+        <v>240</v>
       </c>
       <c r="R6">
         <v>0</v>
@@ -1371,51 +1509,51 @@
         <v>90</v>
       </c>
       <c r="U6">
-        <v>9638</v>
+        <v>6424</v>
       </c>
       <c r="V6" t="s">
-        <v>169</v>
+        <v>209</v>
       </c>
       <c r="W6">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="X6">
-        <v>99</v>
+        <v>728</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="F7" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G7" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="H7" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I7" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="J7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K7">
-        <v>228</v>
+        <v>9</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1427,13 +1565,13 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>142</v>
+        <v>171</v>
       </c>
       <c r="P7">
-        <v>250</v>
+        <v>10</v>
       </c>
       <c r="Q7">
-        <v>388</v>
+        <v>18</v>
       </c>
       <c r="R7">
         <v>0</v>
@@ -1445,16 +1583,16 @@
         <v>90</v>
       </c>
       <c r="U7">
-        <v>15441</v>
+        <v>3947</v>
       </c>
       <c r="V7" t="s">
-        <v>167</v>
+        <v>210</v>
       </c>
       <c r="W7">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="X7">
-        <v>387</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
@@ -1462,37 +1600,37 @@
         <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="F8" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="H8" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I8" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="J8">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K8">
-        <v>102</v>
+        <v>-548</v>
       </c>
       <c r="L8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M8">
         <v>0</v>
@@ -1501,13 +1639,13 @@
         <v>0</v>
       </c>
       <c r="O8" t="s">
-        <v>143</v>
+        <v>172</v>
       </c>
       <c r="P8">
-        <v>150</v>
+        <v>24</v>
       </c>
       <c r="Q8">
-        <v>210</v>
+        <v>36</v>
       </c>
       <c r="R8">
         <v>0</v>
@@ -1519,51 +1657,51 @@
         <v>90</v>
       </c>
       <c r="U8">
-        <v>15134</v>
+        <v>10181</v>
       </c>
       <c r="V8" t="s">
-        <v>170</v>
+        <v>211</v>
       </c>
       <c r="W8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="X8">
-        <v>6</v>
+        <v>30.92</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="F9" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="G9" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="H9" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I9" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="J9">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K9">
-        <v>3</v>
+        <v>133</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -1575,13 +1713,13 @@
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>144</v>
+        <v>173</v>
       </c>
       <c r="P9">
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="Q9">
-        <v>8</v>
+        <v>238</v>
       </c>
       <c r="R9">
         <v>0</v>
@@ -1593,51 +1731,51 @@
         <v>90</v>
       </c>
       <c r="U9">
-        <v>3947</v>
+        <v>15441</v>
       </c>
       <c r="V9" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="W9">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="X9">
-        <v>5</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="F10" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="H10" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I10" t="s">
-        <v>127</v>
+        <v>155</v>
       </c>
       <c r="J10">
         <v>6</v>
       </c>
       <c r="K10">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -1649,13 +1787,13 @@
         <v>0</v>
       </c>
       <c r="O10" t="s">
-        <v>145</v>
+        <v>174</v>
       </c>
       <c r="P10">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="Q10">
-        <v>24</v>
+        <v>102</v>
       </c>
       <c r="R10">
         <v>0</v>
@@ -1667,51 +1805,51 @@
         <v>90</v>
       </c>
       <c r="U10">
-        <v>3947</v>
+        <v>15441</v>
       </c>
       <c r="V10" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="W10">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="X10">
-        <v>9</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="F11" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G11" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="H11" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I11" t="s">
-        <v>127</v>
+        <v>156</v>
       </c>
       <c r="J11">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="K11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1723,13 +1861,13 @@
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>146</v>
+        <v>175</v>
       </c>
       <c r="P11">
-        <v>6</v>
+        <v>0.85399999999999998</v>
       </c>
       <c r="Q11">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="R11">
         <v>0</v>
@@ -1741,69 +1879,69 @@
         <v>90</v>
       </c>
       <c r="U11">
-        <v>3947</v>
+        <v>14718</v>
       </c>
       <c r="V11" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
       <c r="W11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X11">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="F12" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="G12" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="H12" t="s">
+        <v>150</v>
+      </c>
+      <c r="I12" t="s">
+        <v>154</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12">
+        <v>111</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12" t="s">
+        <v>176</v>
+      </c>
+      <c r="P12">
         <v>124</v>
       </c>
-      <c r="I12" t="s">
-        <v>127</v>
-      </c>
-      <c r="J12">
-        <v>6</v>
-      </c>
-      <c r="K12">
-        <v>2</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="O12" t="s">
-        <v>147</v>
-      </c>
-      <c r="P12">
-        <v>6</v>
-      </c>
       <c r="Q12">
-        <v>12</v>
+        <v>196</v>
       </c>
       <c r="R12">
         <v>0</v>
@@ -1815,51 +1953,51 @@
         <v>90</v>
       </c>
       <c r="U12">
-        <v>3947</v>
+        <v>15441</v>
       </c>
       <c r="V12" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="W12">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="X12">
-        <v>24</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
         <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="F13" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="G13" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="H13" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I13" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="J13">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="K13">
-        <v>104</v>
+        <v>158</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -1871,13 +2009,13 @@
         <v>0</v>
       </c>
       <c r="O13" t="s">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="P13">
-        <v>105</v>
+        <v>170</v>
       </c>
       <c r="Q13">
-        <v>165</v>
+        <v>266</v>
       </c>
       <c r="R13">
         <v>0</v>
@@ -1889,52 +2027,52 @@
         <v>90</v>
       </c>
       <c r="U13">
-        <v>6158</v>
+        <v>15441</v>
       </c>
       <c r="V13" t="s">
-        <v>172</v>
+        <v>207</v>
       </c>
       <c r="W13">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="X13">
-        <v>459</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" t="s">
+        <v>123</v>
+      </c>
+      <c r="G14" t="s">
+        <v>134</v>
+      </c>
+      <c r="H14" t="s">
+        <v>150</v>
+      </c>
+      <c r="I14" t="s">
+        <v>157</v>
+      </c>
+      <c r="J14">
+        <v>16</v>
+      </c>
+      <c r="K14">
         <v>27</v>
       </c>
-      <c r="B14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" t="s">
-        <v>55</v>
-      </c>
-      <c r="E14" t="s">
-        <v>86</v>
-      </c>
-      <c r="F14" t="s">
-        <v>107</v>
-      </c>
-      <c r="G14" t="s">
-        <v>113</v>
-      </c>
-      <c r="H14" t="s">
-        <v>124</v>
-      </c>
-      <c r="I14" t="s">
-        <v>127</v>
-      </c>
-      <c r="J14">
-        <v>6</v>
-      </c>
-      <c r="K14">
-        <v>5</v>
-      </c>
       <c r="L14">
         <v>0</v>
       </c>
@@ -1945,13 +2083,13 @@
         <v>0</v>
       </c>
       <c r="O14" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="P14">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="Q14">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="R14">
         <v>0</v>
@@ -1963,51 +2101,51 @@
         <v>90</v>
       </c>
       <c r="U14">
-        <v>6644</v>
+        <v>15134</v>
       </c>
       <c r="V14" t="s">
-        <v>173</v>
+        <v>213</v>
       </c>
       <c r="W14">
         <v>2</v>
       </c>
       <c r="X14">
-        <v>8</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="F15" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="G15" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="H15" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I15" t="s">
-        <v>127</v>
+        <v>154</v>
       </c>
       <c r="J15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K15">
-        <v>183</v>
+        <v>74</v>
       </c>
       <c r="L15">
         <v>0</v>
@@ -2019,13 +2157,13 @@
         <v>0</v>
       </c>
       <c r="O15" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="P15">
-        <v>184</v>
+        <v>80</v>
       </c>
       <c r="Q15">
-        <v>286</v>
+        <v>128</v>
       </c>
       <c r="R15">
         <v>0</v>
@@ -2040,48 +2178,48 @@
         <v>15441</v>
       </c>
       <c r="V15" t="s">
-        <v>167</v>
+        <v>207</v>
       </c>
       <c r="W15">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="X15">
-        <v>387</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F16" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G16" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="H16" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I16" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
       <c r="J16">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K16">
-        <v>67</v>
+        <v>0.81599999999999995</v>
       </c>
       <c r="L16">
         <v>0</v>
@@ -2093,13 +2231,13 @@
         <v>0</v>
       </c>
       <c r="O16" t="s">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="P16">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="Q16">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="R16">
         <v>0</v>
@@ -2111,51 +2249,51 @@
         <v>90</v>
       </c>
       <c r="U16">
-        <v>15134</v>
+        <v>14718</v>
       </c>
       <c r="V16" t="s">
-        <v>170</v>
+        <v>212</v>
       </c>
       <c r="W16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X16">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
         <v>57</v>
       </c>
       <c r="E17" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F17" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G17" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="H17" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I17" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="J17">
-        <v>108</v>
+        <v>6</v>
       </c>
       <c r="K17">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="L17">
         <v>0</v>
@@ -2167,13 +2305,13 @@
         <v>0</v>
       </c>
       <c r="O17" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="P17">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="Q17">
-        <v>174</v>
+        <v>60</v>
       </c>
       <c r="R17">
         <v>0</v>
@@ -2185,16 +2323,16 @@
         <v>90</v>
       </c>
       <c r="U17">
-        <v>5894</v>
+        <v>15441</v>
       </c>
       <c r="V17" t="s">
-        <v>174</v>
+        <v>207</v>
       </c>
       <c r="W17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X17">
-        <v>5</v>
+        <v>330</v>
       </c>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.25">
@@ -2202,37 +2340,37 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D18" t="s">
         <v>58</v>
       </c>
       <c r="E18" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="F18" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="G18" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
       <c r="H18" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I18" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="J18">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K18">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="L18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="M18">
         <v>0</v>
@@ -2241,13 +2379,13 @@
         <v>0</v>
       </c>
       <c r="O18" t="s">
-        <v>152</v>
+        <v>182</v>
       </c>
       <c r="P18">
-        <v>75</v>
+        <v>16</v>
       </c>
       <c r="Q18">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="R18">
         <v>0</v>
@@ -2259,51 +2397,51 @@
         <v>90</v>
       </c>
       <c r="U18">
-        <v>15134</v>
+        <v>9638</v>
       </c>
       <c r="V18" t="s">
-        <v>170</v>
+        <v>214</v>
       </c>
       <c r="W18">
         <v>3</v>
       </c>
       <c r="X18">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D19" t="s">
         <v>59</v>
       </c>
       <c r="E19" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="F19" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="G19" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="H19" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I19" t="s">
-        <v>131</v>
+        <v>158</v>
       </c>
       <c r="J19">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="K19">
-        <v>9</v>
+        <v>191</v>
       </c>
       <c r="L19">
         <v>0</v>
@@ -2315,13 +2453,13 @@
         <v>0</v>
       </c>
       <c r="O19" t="s">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="P19">
-        <v>10</v>
+        <v>192</v>
       </c>
       <c r="Q19">
-        <v>22</v>
+        <v>288</v>
       </c>
       <c r="R19">
         <v>0</v>
@@ -2333,51 +2471,51 @@
         <v>90</v>
       </c>
       <c r="U19">
-        <v>15318</v>
+        <v>7715</v>
       </c>
       <c r="V19" t="s">
-        <v>175</v>
+        <v>215</v>
       </c>
       <c r="W19">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X19">
-        <v>19</v>
+        <v>493.04</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
         <v>60</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="F20" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G20" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="H20" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I20" t="s">
-        <v>131</v>
+        <v>158</v>
       </c>
       <c r="J20">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="K20">
-        <v>221</v>
+        <v>0</v>
       </c>
       <c r="L20">
         <v>0</v>
@@ -2389,13 +2527,13 @@
         <v>0</v>
       </c>
       <c r="O20" t="s">
-        <v>154</v>
+        <v>184</v>
       </c>
       <c r="P20">
-        <v>236</v>
+        <v>40</v>
       </c>
       <c r="Q20">
-        <v>368</v>
+        <v>64</v>
       </c>
       <c r="R20">
         <v>0</v>
@@ -2407,16 +2545,16 @@
         <v>90</v>
       </c>
       <c r="U20">
-        <v>9379</v>
+        <v>10334</v>
       </c>
       <c r="V20" t="s">
-        <v>176</v>
+        <v>216</v>
       </c>
       <c r="W20">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="X20">
-        <v>796</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
@@ -2427,49 +2565,49 @@
         <v>31</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D21" t="s">
         <v>61</v>
       </c>
       <c r="E21" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F21" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G21" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="H21" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I21" t="s">
-        <v>129</v>
+        <v>158</v>
       </c>
       <c r="J21">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="K21">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N21">
         <v>0</v>
       </c>
       <c r="O21" t="s">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="P21">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="Q21">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="R21">
         <v>0</v>
@@ -2481,48 +2619,48 @@
         <v>90</v>
       </c>
       <c r="U21">
-        <v>5894</v>
+        <v>14468</v>
       </c>
       <c r="V21" t="s">
-        <v>174</v>
+        <v>217</v>
       </c>
       <c r="W21">
         <v>2</v>
       </c>
       <c r="X21">
-        <v>38</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D22" t="s">
         <v>62</v>
       </c>
       <c r="E22" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="F22" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G22" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="H22" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I22" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="J22">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -2537,13 +2675,13 @@
         <v>0</v>
       </c>
       <c r="O22" t="s">
-        <v>156</v>
+        <v>186</v>
       </c>
       <c r="P22">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="Q22">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="R22">
         <v>0</v>
@@ -2555,24 +2693,24 @@
         <v>90</v>
       </c>
       <c r="U22">
-        <v>21894</v>
+        <v>17017</v>
       </c>
       <c r="V22" t="s">
-        <v>177</v>
+        <v>218</v>
       </c>
       <c r="W22">
         <v>2</v>
       </c>
       <c r="X22">
-        <v>8</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C23" t="s">
         <v>41</v>
@@ -2581,25 +2719,25 @@
         <v>63</v>
       </c>
       <c r="E23" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F23" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G23" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="H23" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I23" t="s">
-        <v>128</v>
+        <v>48</v>
       </c>
       <c r="J23">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="K23">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L23">
         <v>0</v>
@@ -2611,13 +2749,13 @@
         <v>0</v>
       </c>
       <c r="O23" t="s">
-        <v>157</v>
+        <v>187</v>
       </c>
       <c r="P23">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="Q23">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="R23">
         <v>0</v>
@@ -2629,51 +2767,51 @@
         <v>90</v>
       </c>
       <c r="U23">
-        <v>7995</v>
+        <v>6644</v>
       </c>
       <c r="V23" t="s">
-        <v>178</v>
+        <v>219</v>
       </c>
       <c r="W23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X23">
-        <v>45</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
         <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
         <v>64</v>
       </c>
       <c r="E24" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="F24" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G24" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="H24" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I24" t="s">
-        <v>129</v>
+        <v>48</v>
       </c>
       <c r="J24">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="K24">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -2685,13 +2823,13 @@
         <v>0</v>
       </c>
       <c r="O24" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="P24">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="Q24">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="R24">
         <v>0</v>
@@ -2703,51 +2841,51 @@
         <v>90</v>
       </c>
       <c r="U24">
-        <v>15134</v>
+        <v>6644</v>
       </c>
       <c r="V24" t="s">
-        <v>170</v>
+        <v>219</v>
       </c>
       <c r="W24">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X24">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" t="s">
         <v>65</v>
       </c>
       <c r="E25" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="F25" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G25" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="H25" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I25" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="J25">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="K25">
-        <v>164</v>
+        <v>0</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -2759,13 +2897,13 @@
         <v>0</v>
       </c>
       <c r="O25" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P25">
-        <v>172</v>
+        <v>64</v>
       </c>
       <c r="Q25">
-        <v>268</v>
+        <v>88</v>
       </c>
       <c r="R25">
         <v>0</v>
@@ -2777,51 +2915,51 @@
         <v>90</v>
       </c>
       <c r="U25">
-        <v>15441</v>
+        <v>21220</v>
       </c>
       <c r="V25" t="s">
-        <v>167</v>
+        <v>220</v>
       </c>
       <c r="W25">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="X25">
-        <v>141</v>
+        <v>400</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B26" t="s">
         <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D26" t="s">
         <v>66</v>
       </c>
       <c r="E26" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F26" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G26" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="H26" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I26" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="J26">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K26">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -2833,13 +2971,13 @@
         <v>0</v>
       </c>
       <c r="O26" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="P26">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q26">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="R26">
         <v>0</v>
@@ -2851,51 +2989,51 @@
         <v>90</v>
       </c>
       <c r="U26">
-        <v>15134</v>
+        <v>14468</v>
       </c>
       <c r="V26" t="s">
-        <v>170</v>
+        <v>217</v>
       </c>
       <c r="W26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X26">
-        <v>10</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D27" t="s">
         <v>67</v>
       </c>
       <c r="E27" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="F27" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G27" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="H27" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I27" t="s">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="J27">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="K27">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -2907,13 +3045,13 @@
         <v>0</v>
       </c>
       <c r="O27" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
       <c r="P27">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="Q27">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="R27">
         <v>0</v>
@@ -2925,51 +3063,51 @@
         <v>90</v>
       </c>
       <c r="U27">
-        <v>10181</v>
+        <v>21822</v>
       </c>
       <c r="V27" t="s">
-        <v>179</v>
+        <v>221</v>
       </c>
       <c r="W27">
         <v>2</v>
       </c>
       <c r="X27">
-        <v>76</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C28" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D28" t="s">
         <v>68</v>
       </c>
       <c r="E28" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="F28" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G28" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="H28" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I28" t="s">
-        <v>128</v>
+        <v>161</v>
       </c>
       <c r="J28">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="K28">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="L28">
         <v>0</v>
@@ -2981,13 +3119,13 @@
         <v>0</v>
       </c>
       <c r="O28" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="P28">
-        <v>16</v>
+        <v>66</v>
       </c>
       <c r="Q28">
-        <v>40</v>
+        <v>174</v>
       </c>
       <c r="R28">
         <v>0</v>
@@ -2999,51 +3137,51 @@
         <v>90</v>
       </c>
       <c r="U28">
-        <v>15134</v>
+        <v>5894</v>
       </c>
       <c r="V28" t="s">
-        <v>170</v>
+        <v>222</v>
       </c>
       <c r="W28">
         <v>2</v>
       </c>
       <c r="X28">
-        <v>13</v>
+        <v>30.89</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
         <v>69</v>
       </c>
       <c r="E29" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="F29" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G29" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="H29" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I29" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="J29">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="K29">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="L29">
         <v>0</v>
@@ -3055,13 +3193,13 @@
         <v>0</v>
       </c>
       <c r="O29" t="s">
-        <v>163</v>
+        <v>190</v>
       </c>
       <c r="P29">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="Q29">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="R29">
         <v>0</v>
@@ -3073,51 +3211,51 @@
         <v>90</v>
       </c>
       <c r="U29">
-        <v>12447</v>
+        <v>6424</v>
       </c>
       <c r="V29" t="s">
-        <v>180</v>
+        <v>209</v>
       </c>
       <c r="W29">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X29">
-        <v>69</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B30" t="s">
         <v>31</v>
       </c>
       <c r="C30" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D30" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E30" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="F30" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="G30" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
       <c r="H30" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I30" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="J30">
-        <v>15</v>
+        <v>108</v>
       </c>
       <c r="K30">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L30">
         <v>0</v>
@@ -3129,13 +3267,13 @@
         <v>0</v>
       </c>
       <c r="O30" t="s">
-        <v>137</v>
+        <v>191</v>
       </c>
       <c r="P30">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="Q30">
-        <v>105</v>
+        <v>236</v>
       </c>
       <c r="R30">
         <v>0</v>
@@ -3147,51 +3285,51 @@
         <v>90</v>
       </c>
       <c r="U30">
-        <v>15134</v>
+        <v>11112</v>
       </c>
       <c r="V30" t="s">
-        <v>170</v>
+        <v>223</v>
       </c>
       <c r="W30">
         <v>3</v>
       </c>
       <c r="X30">
-        <v>5</v>
+        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D31" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="E31" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="F31" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G31" t="s">
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="H31" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I31" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="J31">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="K31">
-        <v>12</v>
+        <v>-18</v>
       </c>
       <c r="L31">
         <v>0</v>
@@ -3203,13 +3341,13 @@
         <v>0</v>
       </c>
       <c r="O31" t="s">
-        <v>164</v>
+        <v>192</v>
       </c>
       <c r="P31">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="Q31">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="R31">
         <v>0</v>
@@ -3221,51 +3359,51 @@
         <v>90</v>
       </c>
       <c r="U31">
-        <v>10489</v>
+        <v>10181</v>
       </c>
       <c r="V31" t="s">
-        <v>181</v>
+        <v>211</v>
       </c>
       <c r="W31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X31">
-        <v>12</v>
+        <v>30.92</v>
       </c>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C32" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D32" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E32" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="F32" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="G32" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="H32" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I32" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="J32">
-        <v>480</v>
+        <v>8</v>
       </c>
       <c r="K32">
-        <v>254</v>
+        <v>356</v>
       </c>
       <c r="L32">
         <v>0</v>
@@ -3277,13 +3415,13 @@
         <v>0</v>
       </c>
       <c r="O32" t="s">
-        <v>165</v>
+        <v>193</v>
       </c>
       <c r="P32">
-        <v>288</v>
+        <v>358</v>
       </c>
       <c r="Q32">
-        <v>768</v>
+        <v>558</v>
       </c>
       <c r="R32">
         <v>0</v>
@@ -3295,16 +3433,16 @@
         <v>90</v>
       </c>
       <c r="U32">
-        <v>14200</v>
+        <v>15441</v>
       </c>
       <c r="V32" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="W32">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="X32">
-        <v>23</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.25">
@@ -3312,34 +3450,34 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E33" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="F33" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G33" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="H33" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I33" t="s">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="J33">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="K33">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="L33">
         <v>0</v>
@@ -3351,13 +3489,13 @@
         <v>0</v>
       </c>
       <c r="O33" t="s">
-        <v>166</v>
+        <v>194</v>
       </c>
       <c r="P33">
-        <v>6</v>
+        <v>120</v>
       </c>
       <c r="Q33">
-        <v>16</v>
+        <v>160</v>
       </c>
       <c r="R33">
         <v>0</v>
@@ -3369,16 +3507,16 @@
         <v>90</v>
       </c>
       <c r="U33">
-        <v>21894</v>
+        <v>7995</v>
       </c>
       <c r="V33" t="s">
-        <v>177</v>
+        <v>224</v>
       </c>
       <c r="W33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X33">
-        <v>21</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.25">
@@ -3386,52 +3524,52 @@
         <v>25</v>
       </c>
       <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" t="s">
+        <v>72</v>
+      </c>
+      <c r="E34" t="s">
+        <v>111</v>
+      </c>
+      <c r="F34" t="s">
+        <v>123</v>
+      </c>
+      <c r="G34" t="s">
+        <v>140</v>
+      </c>
+      <c r="H34" t="s">
+        <v>150</v>
+      </c>
+      <c r="I34" t="s">
+        <v>163</v>
+      </c>
+      <c r="J34">
+        <v>10</v>
+      </c>
+      <c r="K34">
+        <v>5</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34">
         <v>30</v>
       </c>
-      <c r="C34" t="s">
-        <v>43</v>
-      </c>
-      <c r="D34" t="s">
-        <v>73</v>
-      </c>
-      <c r="E34" t="s">
-        <v>104</v>
-      </c>
-      <c r="F34" t="s">
-        <v>107</v>
-      </c>
-      <c r="G34" t="s">
-        <v>122</v>
-      </c>
-      <c r="H34" t="s">
-        <v>124</v>
-      </c>
-      <c r="I34" t="s">
-        <v>131</v>
-      </c>
-      <c r="J34">
-        <v>12</v>
-      </c>
-      <c r="K34">
-        <v>0</v>
-      </c>
-      <c r="L34">
-        <v>0</v>
-      </c>
-      <c r="M34">
-        <v>0</v>
-      </c>
-      <c r="N34">
-        <v>0</v>
-      </c>
       <c r="O34" t="s">
-        <v>137</v>
+        <v>195</v>
       </c>
       <c r="P34">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="Q34">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="R34">
         <v>0</v>
@@ -3443,16 +3581,16 @@
         <v>90</v>
       </c>
       <c r="U34">
-        <v>11515</v>
+        <v>2977</v>
       </c>
       <c r="V34" t="s">
-        <v>183</v>
+        <v>225</v>
       </c>
       <c r="W34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X34">
-        <v>53</v>
+        <v>64.900000000000006</v>
       </c>
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.25">
@@ -3460,34 +3598,34 @@
         <v>25</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C35" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E35" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="F35" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G35" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="H35" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="I35" t="s">
-        <v>129</v>
+        <v>158</v>
       </c>
       <c r="J35">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="K35">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="L35">
         <v>0</v>
@@ -3499,13 +3637,13 @@
         <v>0</v>
       </c>
       <c r="O35" t="s">
-        <v>137</v>
+        <v>196</v>
       </c>
       <c r="P35">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="Q35">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="R35">
         <v>0</v>
@@ -3517,20 +3655,834 @@
         <v>90</v>
       </c>
       <c r="U35">
-        <v>16062</v>
+        <v>14671</v>
       </c>
       <c r="V35" t="s">
-        <v>184</v>
+        <v>226</v>
       </c>
       <c r="W35">
         <v>2</v>
       </c>
       <c r="X35">
-        <v>7</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" t="s">
+        <v>42</v>
+      </c>
+      <c r="D36" t="s">
+        <v>74</v>
+      </c>
+      <c r="E36" t="s">
+        <v>113</v>
+      </c>
+      <c r="F36" t="s">
+        <v>123</v>
+      </c>
+      <c r="G36" t="s">
+        <v>142</v>
+      </c>
+      <c r="H36" t="s">
+        <v>150</v>
+      </c>
+      <c r="I36" t="s">
+        <v>156</v>
+      </c>
+      <c r="J36">
+        <v>20</v>
+      </c>
+      <c r="K36">
+        <v>48</v>
+      </c>
+      <c r="L36">
+        <v>0</v>
+      </c>
+      <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36">
+        <v>0</v>
+      </c>
+      <c r="O36" t="s">
+        <v>197</v>
+      </c>
+      <c r="P36">
+        <v>54</v>
+      </c>
+      <c r="Q36">
+        <v>94</v>
+      </c>
+      <c r="R36">
+        <v>0</v>
+      </c>
+      <c r="S36">
+        <v>0</v>
+      </c>
+      <c r="T36">
+        <v>90</v>
+      </c>
+      <c r="U36">
+        <v>16963</v>
+      </c>
+      <c r="V36" t="s">
+        <v>227</v>
+      </c>
+      <c r="W36">
+        <v>3</v>
+      </c>
+      <c r="X36">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" t="s">
+        <v>75</v>
+      </c>
+      <c r="E37" t="s">
+        <v>114</v>
+      </c>
+      <c r="F37" t="s">
+        <v>123</v>
+      </c>
+      <c r="G37" t="s">
+        <v>143</v>
+      </c>
+      <c r="H37" t="s">
+        <v>150</v>
+      </c>
+      <c r="I37" t="s">
+        <v>156</v>
+      </c>
+      <c r="J37">
+        <v>20</v>
+      </c>
+      <c r="K37">
+        <v>15</v>
+      </c>
+      <c r="L37">
+        <v>0</v>
+      </c>
+      <c r="M37">
+        <v>0</v>
+      </c>
+      <c r="N37">
+        <v>0</v>
+      </c>
+      <c r="O37" t="s">
+        <v>198</v>
+      </c>
+      <c r="P37">
+        <v>20</v>
+      </c>
+      <c r="Q37">
+        <v>40</v>
+      </c>
+      <c r="R37">
+        <v>0</v>
+      </c>
+      <c r="S37">
+        <v>0</v>
+      </c>
+      <c r="T37">
+        <v>90</v>
+      </c>
+      <c r="U37">
+        <v>12257</v>
+      </c>
+      <c r="V37" t="s">
+        <v>228</v>
+      </c>
+      <c r="W37">
+        <v>2</v>
+      </c>
+      <c r="X37">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>25</v>
+      </c>
+      <c r="B38" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" t="s">
+        <v>42</v>
+      </c>
+      <c r="D38" t="s">
+        <v>76</v>
+      </c>
+      <c r="E38" t="s">
+        <v>115</v>
+      </c>
+      <c r="F38" t="s">
+        <v>123</v>
+      </c>
+      <c r="G38" t="s">
+        <v>144</v>
+      </c>
+      <c r="H38" t="s">
+        <v>150</v>
+      </c>
+      <c r="I38" t="s">
+        <v>164</v>
+      </c>
+      <c r="J38">
+        <v>50</v>
+      </c>
+      <c r="K38">
+        <v>13</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38">
+        <v>0</v>
+      </c>
+      <c r="O38" t="s">
+        <v>199</v>
+      </c>
+      <c r="P38">
+        <v>30</v>
+      </c>
+      <c r="Q38">
+        <v>80</v>
+      </c>
+      <c r="R38">
+        <v>0</v>
+      </c>
+      <c r="S38">
+        <v>0</v>
+      </c>
+      <c r="T38">
+        <v>90</v>
+      </c>
+      <c r="U38">
+        <v>10189</v>
+      </c>
+      <c r="V38" t="s">
+        <v>229</v>
+      </c>
+      <c r="W38">
+        <v>2</v>
+      </c>
+      <c r="X38">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B39" t="s">
+        <v>32</v>
+      </c>
+      <c r="C39" t="s">
+        <v>42</v>
+      </c>
+      <c r="D39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E39" t="s">
+        <v>116</v>
+      </c>
+      <c r="F39" t="s">
+        <v>123</v>
+      </c>
+      <c r="G39" t="s">
+        <v>145</v>
+      </c>
+      <c r="H39" t="s">
+        <v>150</v>
+      </c>
+      <c r="I39" t="s">
+        <v>160</v>
+      </c>
+      <c r="J39">
+        <v>72</v>
+      </c>
+      <c r="K39">
+        <v>59</v>
+      </c>
+      <c r="L39">
+        <v>0</v>
+      </c>
+      <c r="M39">
+        <v>0</v>
+      </c>
+      <c r="N39">
+        <v>0</v>
+      </c>
+      <c r="O39" t="s">
+        <v>200</v>
+      </c>
+      <c r="P39">
+        <v>62</v>
+      </c>
+      <c r="Q39">
+        <v>134</v>
+      </c>
+      <c r="R39">
+        <v>0</v>
+      </c>
+      <c r="S39">
+        <v>0</v>
+      </c>
+      <c r="T39">
+        <v>90</v>
+      </c>
+      <c r="U39">
+        <v>13838</v>
+      </c>
+      <c r="V39" t="s">
+        <v>230</v>
+      </c>
+      <c r="W39">
+        <v>2</v>
+      </c>
+      <c r="X39">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>25</v>
+      </c>
+      <c r="B40" t="s">
+        <v>32</v>
+      </c>
+      <c r="C40" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" t="s">
+        <v>78</v>
+      </c>
+      <c r="E40" t="s">
+        <v>117</v>
+      </c>
+      <c r="F40" t="s">
+        <v>123</v>
+      </c>
+      <c r="G40" t="s">
+        <v>126</v>
+      </c>
+      <c r="H40" t="s">
+        <v>150</v>
+      </c>
+      <c r="I40" t="s">
+        <v>151</v>
+      </c>
+      <c r="J40">
+        <v>12</v>
+      </c>
+      <c r="K40">
+        <v>6</v>
+      </c>
+      <c r="L40">
+        <v>0</v>
+      </c>
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40" t="s">
+        <v>201</v>
+      </c>
+      <c r="P40">
+        <v>12</v>
+      </c>
+      <c r="Q40">
+        <v>24</v>
+      </c>
+      <c r="R40">
+        <v>0</v>
+      </c>
+      <c r="S40">
+        <v>0</v>
+      </c>
+      <c r="T40">
+        <v>90</v>
+      </c>
+      <c r="U40">
+        <v>10683</v>
+      </c>
+      <c r="V40" t="s">
+        <v>231</v>
+      </c>
+      <c r="W40">
+        <v>2</v>
+      </c>
+      <c r="X40">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>26</v>
+      </c>
+      <c r="B41" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" t="s">
+        <v>42</v>
+      </c>
+      <c r="D41" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41" t="s">
+        <v>118</v>
+      </c>
+      <c r="F41" t="s">
+        <v>123</v>
+      </c>
+      <c r="G41" t="s">
+        <v>146</v>
+      </c>
+      <c r="H41" t="s">
+        <v>150</v>
+      </c>
+      <c r="I41" t="s">
+        <v>158</v>
+      </c>
+      <c r="J41">
+        <v>24</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41">
+        <v>0</v>
+      </c>
+      <c r="O41" t="s">
+        <v>166</v>
+      </c>
+      <c r="P41">
+        <v>16</v>
+      </c>
+      <c r="Q41">
+        <v>40</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
+      </c>
+      <c r="S41">
+        <v>0</v>
+      </c>
+      <c r="T41">
+        <v>90</v>
+      </c>
+      <c r="U41">
+        <v>14469</v>
+      </c>
+      <c r="V41" t="s">
+        <v>232</v>
+      </c>
+      <c r="W41">
+        <v>2</v>
+      </c>
+      <c r="X41">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>25</v>
+      </c>
+      <c r="B42" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" t="s">
+        <v>43</v>
+      </c>
+      <c r="D42" t="s">
+        <v>80</v>
+      </c>
+      <c r="E42" t="s">
+        <v>119</v>
+      </c>
+      <c r="F42" t="s">
+        <v>123</v>
+      </c>
+      <c r="G42" t="s">
+        <v>147</v>
+      </c>
+      <c r="H42" t="s">
+        <v>150</v>
+      </c>
+      <c r="I42" t="s">
+        <v>163</v>
+      </c>
+      <c r="J42">
+        <v>10</v>
+      </c>
+      <c r="K42">
+        <v>19</v>
+      </c>
+      <c r="L42">
+        <v>0</v>
+      </c>
+      <c r="M42">
+        <v>0</v>
+      </c>
+      <c r="N42">
+        <v>0</v>
+      </c>
+      <c r="O42" t="s">
+        <v>153</v>
+      </c>
+      <c r="P42">
+        <v>20</v>
+      </c>
+      <c r="Q42">
+        <v>30</v>
+      </c>
+      <c r="R42">
+        <v>0</v>
+      </c>
+      <c r="S42">
+        <v>0</v>
+      </c>
+      <c r="T42">
+        <v>90</v>
+      </c>
+      <c r="U42">
+        <v>10153</v>
+      </c>
+      <c r="V42" t="s">
+        <v>233</v>
+      </c>
+      <c r="W42">
+        <v>2</v>
+      </c>
+      <c r="X42">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>25</v>
+      </c>
+      <c r="B43" t="s">
+        <v>32</v>
+      </c>
+      <c r="C43" t="s">
+        <v>43</v>
+      </c>
+      <c r="D43" t="s">
+        <v>81</v>
+      </c>
+      <c r="E43" t="s">
+        <v>120</v>
+      </c>
+      <c r="F43" t="s">
+        <v>123</v>
+      </c>
+      <c r="G43" t="s">
+        <v>147</v>
+      </c>
+      <c r="H43" t="s">
+        <v>150</v>
+      </c>
+      <c r="I43" t="s">
+        <v>155</v>
+      </c>
+      <c r="J43">
+        <v>6</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+      <c r="L43">
+        <v>0</v>
+      </c>
+      <c r="M43">
+        <v>0</v>
+      </c>
+      <c r="N43">
+        <v>0</v>
+      </c>
+      <c r="O43" t="s">
+        <v>202</v>
+      </c>
+      <c r="P43">
+        <v>18</v>
+      </c>
+      <c r="Q43">
+        <v>30</v>
+      </c>
+      <c r="R43">
+        <v>0</v>
+      </c>
+      <c r="S43">
+        <v>0</v>
+      </c>
+      <c r="T43">
+        <v>90</v>
+      </c>
+      <c r="U43">
+        <v>15134</v>
+      </c>
+      <c r="V43" t="s">
+        <v>213</v>
+      </c>
+      <c r="W43">
+        <v>5</v>
+      </c>
+      <c r="X43">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>25</v>
+      </c>
+      <c r="B44" t="s">
+        <v>32</v>
+      </c>
+      <c r="C44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" t="s">
+        <v>82</v>
+      </c>
+      <c r="E44" t="s">
+        <v>121</v>
+      </c>
+      <c r="F44" t="s">
+        <v>123</v>
+      </c>
+      <c r="G44" t="s">
+        <v>148</v>
+      </c>
+      <c r="H44" t="s">
+        <v>150</v>
+      </c>
+      <c r="I44" t="s">
+        <v>157</v>
+      </c>
+      <c r="J44">
+        <v>16</v>
+      </c>
+      <c r="K44">
+        <v>9</v>
+      </c>
+      <c r="L44">
+        <v>0</v>
+      </c>
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44">
+        <v>0</v>
+      </c>
+      <c r="O44" t="s">
+        <v>203</v>
+      </c>
+      <c r="P44">
+        <v>10</v>
+      </c>
+      <c r="Q44">
+        <v>26</v>
+      </c>
+      <c r="R44">
+        <v>0</v>
+      </c>
+      <c r="S44">
+        <v>0</v>
+      </c>
+      <c r="T44">
+        <v>90</v>
+      </c>
+      <c r="U44">
+        <v>16963</v>
+      </c>
+      <c r="V44" t="s">
+        <v>227</v>
+      </c>
+      <c r="W44">
+        <v>2</v>
+      </c>
+      <c r="X44">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" t="s">
+        <v>81</v>
+      </c>
+      <c r="E45" t="s">
+        <v>120</v>
+      </c>
+      <c r="F45" t="s">
+        <v>123</v>
+      </c>
+      <c r="G45" t="s">
+        <v>147</v>
+      </c>
+      <c r="H45" t="s">
+        <v>150</v>
+      </c>
+      <c r="I45" t="s">
+        <v>155</v>
+      </c>
+      <c r="J45">
+        <v>6</v>
+      </c>
+      <c r="K45">
+        <v>12</v>
+      </c>
+      <c r="L45">
+        <v>0</v>
+      </c>
+      <c r="M45">
+        <v>0</v>
+      </c>
+      <c r="N45">
+        <v>0</v>
+      </c>
+      <c r="O45" t="s">
+        <v>204</v>
+      </c>
+      <c r="P45">
+        <v>14</v>
+      </c>
+      <c r="Q45">
+        <v>20</v>
+      </c>
+      <c r="R45">
+        <v>0</v>
+      </c>
+      <c r="S45">
+        <v>0</v>
+      </c>
+      <c r="T45">
+        <v>90</v>
+      </c>
+      <c r="U45">
+        <v>15134</v>
+      </c>
+      <c r="V45" t="s">
+        <v>213</v>
+      </c>
+      <c r="W45">
+        <v>2</v>
+      </c>
+      <c r="X45">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" t="s">
+        <v>30</v>
+      </c>
+      <c r="C46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E46" t="s">
+        <v>122</v>
+      </c>
+      <c r="F46" t="s">
+        <v>123</v>
+      </c>
+      <c r="G46" t="s">
+        <v>149</v>
+      </c>
+      <c r="H46" t="s">
+        <v>150</v>
+      </c>
+      <c r="I46" t="s">
+        <v>153</v>
+      </c>
+      <c r="J46">
+        <v>4</v>
+      </c>
+      <c r="K46">
+        <v>11</v>
+      </c>
+      <c r="L46">
+        <v>0</v>
+      </c>
+      <c r="M46">
+        <v>24</v>
+      </c>
+      <c r="N46">
+        <v>0</v>
+      </c>
+      <c r="O46" t="s">
+        <v>205</v>
+      </c>
+      <c r="P46">
+        <v>36</v>
+      </c>
+      <c r="Q46">
+        <v>48</v>
+      </c>
+      <c r="R46">
+        <v>0</v>
+      </c>
+      <c r="S46">
+        <v>0</v>
+      </c>
+      <c r="T46">
+        <v>90</v>
+      </c>
+      <c r="U46">
+        <v>6424</v>
+      </c>
+      <c r="V46" t="s">
+        <v>209</v>
+      </c>
+      <c r="W46">
+        <v>4</v>
+      </c>
+      <c r="X46">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X35" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:X46" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>